<commit_message>
Fix EBITDA interest double count and EV securities/debt
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015e6JuRwZeu9ySdnBQS2F4f
</commit_message>
<xml_diff>
--- a/template/epv_template.xlsx
+++ b/template/epv_template.xlsx
@@ -15388,48 +15388,40 @@
       <c r="P12" s="325"/>
     </row>
     <row r="13" spans="2:16" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B13" s="180" t="s">
-        <v>90</v>
+      <c r="B13" s="180" t="inlineStr">
+        <is>
+          <t>Less: Cash + securities</t>
+        </is>
       </c>
       <c r="D13" s="17">
-        <f>D53</f>
-        <v>0</v>
+        <f>D53+D59</f>
       </c>
       <c r="E13" s="18">
-        <f>E53</f>
-        <v>0</v>
+        <f>E53+E59</f>
       </c>
       <c r="F13" s="17">
-        <f t="shared" ref="F13:I13" si="5">F53</f>
-        <v>0</v>
+        <f>F53+F59</f>
       </c>
       <c r="G13" s="18">
-        <f t="shared" si="5"/>
-        <v>0</v>
+        <f>G53+G59</f>
       </c>
       <c r="H13" s="17">
-        <f t="shared" si="5"/>
-        <v>0</v>
+        <f>H53+H59</f>
       </c>
       <c r="I13" s="18">
-        <f t="shared" si="5"/>
-        <v>0</v>
+        <f>I53+I59</f>
       </c>
       <c r="J13" s="183">
-        <f t="shared" ref="J13:K13" si="6">J53</f>
-        <v>0</v>
+        <f>J53+J59</f>
       </c>
       <c r="K13" s="18">
-        <f t="shared" si="6"/>
-        <v>0</v>
+        <f>K53+K59</f>
       </c>
       <c r="L13" s="17">
-        <f t="shared" ref="L13" si="7">L53</f>
-        <v>0</v>
+        <f>L53+L59</f>
       </c>
       <c r="M13" s="18">
-        <f t="shared" ref="M13" si="8">M53</f>
-        <v>0</v>
+        <f>M53+M59</f>
       </c>
       <c r="N13" s="183"/>
       <c r="O13" s="324"/>
@@ -16448,8 +16440,10 @@
       <c r="N52" s="35"/>
     </row>
     <row r="53" spans="2:15" ht="16.149999999999999" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.25">
-      <c r="B53" s="93" t="s">
-        <v>23</v>
+      <c r="B53" s="93" t="inlineStr">
+        <is>
+          <t>Cash, Equivalents + Current Securities</t>
+        </is>
       </c>
       <c r="D53" s="36"/>
       <c r="E53" s="67"/>
@@ -16550,7 +16544,11 @@
       <c r="O58" s="36"/>
     </row>
     <row r="59" spans="2:15" ht="16.149999999999999" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.25">
-      <c r="B59" s="11"/>
+      <c r="B59" s="93" t="inlineStr">
+        <is>
+          <t>Non-current marketable securities</t>
+        </is>
+      </c>
       <c r="D59" s="303"/>
       <c r="E59" s="67"/>
       <c r="F59" s="36"/>
@@ -16646,6 +16644,11 @@
       <c r="O62" s="36"/>
     </row>
     <row r="63" spans="2:15" ht="16.149999999999999" customHeight="1" outlineLevel="2" x14ac:dyDescent="0.25">
+      <c r="B63" s="93" t="inlineStr">
+        <is>
+          <t>  of which: current debt + current op. lease</t>
+        </is>
+      </c>
       <c r="D63" s="303"/>
       <c r="E63" s="67"/>
       <c r="F63" s="36"/>
@@ -16660,8 +16663,10 @@
       <c r="O63" s="36"/>
     </row>
     <row r="64" spans="2:15" ht="16.149999999999999" customHeight="1" outlineLevel="2" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B64" s="295" t="s">
-        <v>111</v>
+      <c r="B64" s="295" t="inlineStr">
+        <is>
+          <t>Total Debt + Operating Leases</t>
+        </is>
       </c>
       <c r="D64" s="303"/>
       <c r="E64" s="67"/>
@@ -17058,48 +17063,40 @@
       <c r="N77" s="43"/>
     </row>
     <row r="78" spans="2:16" ht="16.149999999999999" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.25">
-      <c r="B78" s="258" t="s">
-        <v>17</v>
+      <c r="B78" s="258" t="inlineStr">
+        <is>
+          <t>Less: Interest and other income</t>
+        </is>
       </c>
       <c r="D78" s="306">
-        <f t="shared" ref="D78:I78" si="72">+D41</f>
-        <v>0</v>
+        <f>-D41</f>
       </c>
       <c r="E78" s="69">
-        <f t="shared" si="72"/>
-        <v>0</v>
+        <f>-E41</f>
       </c>
       <c r="F78" s="68">
-        <f t="shared" si="72"/>
-        <v>0</v>
+        <f>-F41</f>
       </c>
       <c r="G78" s="69">
-        <f t="shared" si="72"/>
-        <v>0</v>
+        <f>-G41</f>
       </c>
       <c r="H78" s="68">
-        <f t="shared" si="72"/>
-        <v>0</v>
+        <f>-H41</f>
       </c>
       <c r="I78" s="69">
-        <f t="shared" si="72"/>
-        <v>0</v>
+        <f>-I41</f>
       </c>
       <c r="J78" s="68">
-        <f t="shared" ref="J78:K78" si="73">+J41</f>
-        <v>0</v>
+        <f>-J41</f>
       </c>
       <c r="K78" s="69">
-        <f t="shared" si="73"/>
-        <v>0</v>
+        <f>-K41</f>
       </c>
       <c r="L78" s="68">
-        <f t="shared" ref="L78" si="74">+L41</f>
-        <v>0</v>
+        <f>-L41</f>
       </c>
       <c r="M78" s="69">
-        <f t="shared" ref="M78" si="75">+M41</f>
-        <v>0</v>
+        <f>-M41</f>
       </c>
       <c r="N78" s="68"/>
     </row>
@@ -18593,48 +18590,40 @@
       <c r="P127" s="112"/>
     </row>
     <row r="128" spans="2:16" ht="16.149999999999999" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.25">
-      <c r="B128" s="307" t="s">
-        <v>65</v>
+      <c r="B128" s="307" t="inlineStr">
+        <is>
+          <t>    Current Liabilities (ex debt and leases)</t>
+        </is>
       </c>
       <c r="D128" s="43">
-        <f t="shared" ref="D128:I128" si="167">+D62</f>
-        <v>0</v>
+        <f>+D62-D63</f>
       </c>
       <c r="E128" s="62">
-        <f t="shared" si="167"/>
-        <v>0</v>
+        <f>+E62-E63</f>
       </c>
       <c r="F128" s="43">
-        <f t="shared" si="167"/>
-        <v>0</v>
+        <f>+F62-F63</f>
       </c>
       <c r="G128" s="62">
-        <f t="shared" si="167"/>
-        <v>0</v>
+        <f>+G62-G63</f>
       </c>
       <c r="H128" s="43">
-        <f t="shared" si="167"/>
-        <v>0</v>
+        <f>+H62-H63</f>
       </c>
       <c r="I128" s="62">
-        <f t="shared" si="167"/>
-        <v>0</v>
+        <f>+I62-I63</f>
       </c>
       <c r="J128" s="43">
-        <f t="shared" ref="J128:K128" si="168">+J62</f>
-        <v>0</v>
+        <f>+J62-J63</f>
       </c>
       <c r="K128" s="62">
-        <f t="shared" si="168"/>
-        <v>0</v>
+        <f>+K62-K63</f>
       </c>
       <c r="L128" s="43">
-        <f t="shared" ref="L128" si="169">+L62</f>
-        <v>0</v>
+        <f>+L62-L63</f>
       </c>
       <c r="M128" s="62">
-        <f t="shared" ref="M128" si="170">+M62</f>
-        <v>0</v>
+        <f>+M62-M63</f>
       </c>
       <c r="N128" s="43"/>
       <c r="P128" s="112"/>

</xml_diff>